<commit_message>
new commit -- 31st july 2026
</commit_message>
<xml_diff>
--- a/Conditional_Formatting_Practice.xlsx
+++ b/Conditional_Formatting_Practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dmart_sales_7_9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4650CA88-B45F-4997-96FA-FF72D971833B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CAD05D-6D0F-43EB-A5BC-3509862A4ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="816" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conditional_Formatting_Practice" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="305">
   <si>
     <t>Employee ID</t>
   </si>
@@ -289,9 +289,6 @@
     <t>Category</t>
   </si>
   <si>
-    <t>Order Text</t>
-  </si>
-  <si>
     <t>RAHUL@gmail.com</t>
   </si>
   <si>
@@ -892,30 +889,6 @@
     <t>&amp;</t>
   </si>
   <si>
-    <t>F name</t>
-  </si>
-  <si>
-    <t>L name</t>
-  </si>
-  <si>
-    <t>M name</t>
-  </si>
-  <si>
-    <t>Nikhil</t>
-  </si>
-  <si>
-    <t>Shelar</t>
-  </si>
-  <si>
-    <t>textjoin func</t>
-  </si>
-  <si>
-    <t>salman</t>
-  </si>
-  <si>
-    <t>Person A</t>
-  </si>
-  <si>
     <t>average func</t>
   </si>
   <si>
@@ -962,6 +935,60 @@
   </si>
   <si>
     <t>null</t>
+  </si>
+  <si>
+    <t>Order ID</t>
+  </si>
+  <si>
+    <t>aa</t>
+  </si>
+  <si>
+    <t>aaa</t>
+  </si>
+  <si>
+    <t>aaaa</t>
+  </si>
+  <si>
+    <t>bbbb</t>
+  </si>
+  <si>
+    <t>cccccc</t>
+  </si>
+  <si>
+    <t>left</t>
+  </si>
+  <si>
+    <t>right</t>
+  </si>
+  <si>
+    <t>mid</t>
+  </si>
+  <si>
+    <t>len</t>
+  </si>
+  <si>
+    <t>trim</t>
+  </si>
+  <si>
+    <t>upper</t>
+  </si>
+  <si>
+    <t>lower</t>
+  </si>
+  <si>
+    <t>proper</t>
+  </si>
+  <si>
+    <t>find</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>concat</t>
+  </si>
+  <si>
+    <t>textjoin</t>
   </si>
 </sst>
 </file>
@@ -2030,28 +2057,28 @@
         <v>9</v>
       </c>
       <c r="Z1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AA1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AB1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AH1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AO1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AP1" t="s">
+        <v>187</v>
+      </c>
+      <c r="AQ1" t="s">
         <v>188</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>189</v>
       </c>
       <c r="AY1">
         <v>1</v>
@@ -2101,16 +2128,16 @@
         <v>1</v>
       </c>
       <c r="AA2" t="s">
+        <v>175</v>
+      </c>
+      <c r="AB2" t="s">
         <v>176</v>
       </c>
-      <c r="AB2" t="s">
-        <v>177</v>
-      </c>
       <c r="AG2" t="s">
+        <v>182</v>
+      </c>
+      <c r="AH2" t="s">
         <v>183</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>184</v>
       </c>
       <c r="AP2">
         <v>55</v>
@@ -2163,16 +2190,16 @@
         <v>2</v>
       </c>
       <c r="AA3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB3" t="s">
         <v>178</v>
       </c>
-      <c r="AB3" t="s">
-        <v>179</v>
-      </c>
       <c r="AG3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AH3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AP3">
         <v>51</v>
@@ -2225,16 +2252,16 @@
         <v>3</v>
       </c>
       <c r="AA4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AB4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AG4" t="s">
+        <v>184</v>
+      </c>
+      <c r="AH4" t="s">
         <v>185</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>186</v>
       </c>
       <c r="AP4">
         <v>12</v>
@@ -2287,16 +2314,16 @@
         <v>4</v>
       </c>
       <c r="AA5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AB5" t="s">
         <v>181</v>
       </c>
-      <c r="AB5" t="s">
-        <v>182</v>
-      </c>
       <c r="AG5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AH5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AP5">
         <v>13</v>
@@ -2728,12 +2755,12 @@
     </row>
     <row r="32" spans="5:18" x14ac:dyDescent="0.35">
       <c r="G32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="5:7" x14ac:dyDescent="0.35">
       <c r="G33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="5:7" x14ac:dyDescent="0.35">
@@ -2819,21 +2846,21 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="31" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>139</v>
       </c>
       <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="34" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B2" s="34" t="s">
         <v>52</v>
@@ -2845,24 +2872,24 @@
         <v>42000</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B3" s="34" t="s">
         <v>54</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D3" s="34">
         <v>50000</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H3">
         <f>VLOOKUP("Aman",B1:D6,3,FALSE)</f>
@@ -2875,7 +2902,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="34" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B4" s="34" t="s">
         <v>14</v>
@@ -2889,7 +2916,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="34" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B5" s="34" t="s">
         <v>17</v>
@@ -2903,7 +2930,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B6" s="34" t="s">
         <v>34</v>
@@ -2917,29 +2944,29 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="G10" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="H12" s="31" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J12" s="33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K12" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="L12" s="33" t="s">
         <v>148</v>
-      </c>
-      <c r="L12" s="33" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="H13" s="31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I13" s="34" t="s">
         <v>17</v>
@@ -2956,7 +2983,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="H14" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I14" s="34">
         <v>35000</v>
@@ -3030,7 +3057,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="45" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -3065,7 +3092,7 @@
         <v>13</v>
       </c>
       <c r="M2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
@@ -3100,7 +3127,7 @@
         <v>16</v>
       </c>
       <c r="M3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -3135,7 +3162,7 @@
         <v>20</v>
       </c>
       <c r="M4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -3170,7 +3197,7 @@
         <v>23</v>
       </c>
       <c r="M5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
@@ -3205,7 +3232,7 @@
         <v>26</v>
       </c>
       <c r="M6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -3376,12 +3403,12 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="E13" s="43" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="E14" s="43" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F14">
         <f>SUM(F2:F11)</f>
@@ -3390,7 +3417,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="E15" s="43" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F15">
         <f>AVERAGE(F2:F11)</f>
@@ -3399,7 +3426,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="E16" s="43" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F16">
         <f>MIN(F2:F11)</f>
@@ -3408,7 +3435,7 @@
     </row>
     <row r="17" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E17" s="43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F17">
         <f>MAX(F2:F11)</f>
@@ -3417,7 +3444,7 @@
     </row>
     <row r="18" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E18" s="43" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F18">
         <f>COUNT(F2:F11)</f>
@@ -3437,18 +3464,18 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" t="s">
         <v>196</v>
       </c>
-      <c r="B1" t="s">
-        <v>197</v>
-      </c>
       <c r="E1" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B2">
         <v>197</v>
@@ -3458,12 +3485,12 @@
         <v>197</v>
       </c>
       <c r="E2" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B3">
         <v>144</v>
@@ -3473,12 +3500,12 @@
         <v>144</v>
       </c>
       <c r="E3" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B4">
         <v>139</v>
@@ -3488,27 +3515,27 @@
         <v>139</v>
       </c>
       <c r="E4" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="B5" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C5">
         <f>IF(B5="Null",$B$11,B5)</f>
         <v>161</v>
       </c>
       <c r="E5" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="B6">
         <v>160</v>
@@ -3518,12 +3545,12 @@
         <v>160</v>
       </c>
       <c r="E6" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="B7">
         <v>144</v>
@@ -3533,27 +3560,27 @@
         <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="B8" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
         <v>161</v>
       </c>
       <c r="E8" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B9">
         <v>182</v>
@@ -3565,10 +3592,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="B10" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
@@ -3649,7 +3676,7 @@
         <v>1</v>
       </c>
       <c r="V1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
@@ -3936,10 +3963,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>167</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>168</v>
       </c>
       <c r="D1">
         <v>0</v>
@@ -3961,7 +3988,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D2">
         <v>3</v>
@@ -3983,7 +4010,7 @@
         <v>#N/A</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3">
@@ -4006,7 +4033,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -4025,10 +4052,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -4050,7 +4077,7 @@
         <v>#NAME?</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -4072,7 +4099,7 @@
         <v>#NUM!</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -4100,7 +4127,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AH10"/>
+  <dimension ref="A1:AH15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.6328125" bestFit="1" customWidth="1"/>
@@ -4113,7 +4140,7 @@
     <col min="8" max="8" width="8.08984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.26953125" customWidth="1"/>
+    <col min="11" max="11" width="16.36328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="24.1796875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.7265625" customWidth="1"/>
@@ -4139,70 +4166,70 @@
         <v>70</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>71</v>
+        <v>287</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>90</v>
-      </c>
       <c r="R1" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S1" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="Y1" t="s">
+        <v>122</v>
+      </c>
+      <c r="Z1" t="s">
         <v>123</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>124</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>125</v>
       </c>
-      <c r="AB1" t="s">
-        <v>126</v>
-      </c>
       <c r="AC1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AE1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AF1" t="str">
         <f>MID(AE1,(FIND(" ",AE1,1)),5)</f>
@@ -4215,28 +4242,28 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="E2" t="str">
-        <f>LEFT(A2,5)</f>
-        <v>rahul</v>
+        <f>LEFT(A2,3)</f>
+        <v>rah</v>
       </c>
       <c r="F2" t="str">
-        <f>RIGHT(A2,6)</f>
-        <v xml:space="preserve">ma    </v>
+        <f>RIGHT(D2,5)</f>
+        <v>12345</v>
       </c>
       <c r="G2" t="str">
-        <f>MID(A2,2,4)</f>
-        <v>ahul</v>
+        <f>MID(C2,3,3)</f>
+        <v>ec_</v>
       </c>
       <c r="H2">
         <f>LEN(A2)</f>
@@ -4251,56 +4278,60 @@
         <v>RAHUL SHARMA</v>
       </c>
       <c r="K2" t="str">
-        <f>LOWER(J2)</f>
-        <v>rahul sharma</v>
+        <f>LOWER(B2)</f>
+        <v>rahul@gmail.com</v>
       </c>
       <c r="L2" t="str">
-        <f>PROPER(K2)</f>
+        <f>PROPER(I2)</f>
         <v>Rahul Sharma</v>
       </c>
       <c r="M2" t="str">
-        <f>_xlfn.CONCAT(L2," - ",D2)</f>
-        <v>Rahul Sharma - Order-ID:12345</v>
+        <f>_xlfn.CONCAT(L2," \ ",C2)</f>
+        <v>Rahul Sharma \ elec_mobile</v>
       </c>
       <c r="O2">
-        <f>FIND("ID",D2)</f>
-        <v>7</v>
+        <f>FIND("@",K2)</f>
+        <v>6</v>
       </c>
       <c r="P2">
-        <f>SEARCH("Id",D2)</f>
-        <v>7</v>
+        <f>SEARCH("r",L2)</f>
+        <v>1</v>
       </c>
       <c r="Q2" t="str">
-        <f>SUBSTITUTE(M2,"Order-ID", "")</f>
-        <v>Rahul Sharma - :12345</v>
+        <f>SUBSTITUTE(D2,"Order-", "")</f>
+        <v>ID:12345</v>
+      </c>
+      <c r="R2" t="str">
+        <f>REPLACE(Q2,1,3,L2)</f>
+        <v>Rahul Sharma12345</v>
       </c>
       <c r="U2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="V2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="W2" t="str">
         <f>U2&amp;" "&amp;V2</f>
         <v>Ansari Tarique</v>
       </c>
       <c r="Y2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Z2">
         <v>10</v>
       </c>
       <c r="AA2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AB2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AC2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AE2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AF2" t="str">
         <f>MID(AE2,(FIND(" ",AE2,1)),5)</f>
@@ -4309,28 +4340,28 @@
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="E3" t="str">
-        <f>LEFT(A3,5)</f>
-        <v>aisha</v>
+        <f>LEFT(A3,3)</f>
+        <v>ais</v>
       </c>
       <c r="F3" t="str">
-        <f>RIGHT(A3,6)</f>
-        <v>a Khan</v>
+        <f>RIGHT(D3,5)</f>
+        <v>67890</v>
       </c>
       <c r="G3" t="str">
-        <f>MID(A3,7,6)</f>
-        <v>Khan</v>
+        <f>MID(C3,3,3)</f>
+        <v>me_</v>
       </c>
       <c r="H3">
         <f>LEN(A3)</f>
@@ -4345,87 +4376,149 @@
         <v>AISHA KHAN</v>
       </c>
       <c r="K3" t="str">
-        <f>LOWER(J3)</f>
-        <v>aisha khan</v>
+        <f>LOWER(B3)</f>
+        <v>aisha@yahoo.com</v>
       </c>
       <c r="L3" t="str">
-        <f>PROPER(K3)</f>
+        <f>PROPER(I3)</f>
         <v>Aisha Khan</v>
       </c>
       <c r="M3" t="str">
-        <f>_xlfn.CONCAT(L3," - ",D3)</f>
-        <v>Aisha Khan - Order-ID:67890</v>
-      </c>
-      <c r="O3" t="e">
-        <f>FIND("khan",A3)</f>
+        <f>_xlfn.CONCAT(L3," \ ",C3)</f>
+        <v>Aisha Khan \ home_appliance</v>
+      </c>
+      <c r="O3">
+        <f>FIND("@",K3)</f>
+        <v>6</v>
+      </c>
+      <c r="P3" t="e">
+        <f>SEARCH("r",L3)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P3">
-        <f>SEARCH("Id",D3)</f>
-        <v>7</v>
-      </c>
       <c r="Q3" t="str">
-        <f>SUBSTITUTE(M3,"Order-ID", "")</f>
-        <v>Aisha Khan - :67890</v>
+        <f>SUBSTITUTE(D3,"Order-", "")</f>
+        <v>ID:67890</v>
+      </c>
+      <c r="R3" t="str">
+        <f>REPLACE(Q3,1,3,L3)</f>
+        <v>Aisha Khan67890</v>
       </c>
       <c r="Y3" t="s">
+        <v>128</v>
+      </c>
+      <c r="AA3" t="s">
         <v>129</v>
       </c>
-      <c r="AA3" t="s">
-        <v>130</v>
-      </c>
       <c r="AB3" t="s">
-        <v>132</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>294</v>
+      </c>
+      <c r="K5" t="s">
+        <v>266</v>
+      </c>
+      <c r="L5" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>272</v>
-      </c>
-      <c r="B6" t="s">
-        <v>274</v>
-      </c>
-      <c r="C6" t="s">
-        <v>273</v>
-      </c>
-      <c r="D6" t="s">
-        <v>277</v>
+        <v>295</v>
+      </c>
+      <c r="K6" t="str">
+        <f>K5&amp;L5</f>
+        <v>TariqueAnsari</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>275</v>
-      </c>
-      <c r="C7" t="s">
-        <v>276</v>
-      </c>
-      <c r="D7" t="str">
-        <f>_xlfn.TEXTJOIN(" - ",TRUE,A7,B7,C7)</f>
-        <v>Neha - Nikhil - Shelar</v>
+        <v>296</v>
+      </c>
+      <c r="K7" t="str">
+        <f>K5&amp; " " &amp;L5</f>
+        <v>Tarique Ansari</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>278</v>
-      </c>
-      <c r="C8" t="s">
-        <v>241</v>
-      </c>
-      <c r="D8" t="str">
-        <f>_xlfn.TEXTJOIN(" - ",TRUE,A8,B8,C8)</f>
-        <v>salman - Khan</v>
+        <v>297</v>
+      </c>
+      <c r="K8" t="str">
+        <f>K5&amp;L5</f>
+        <v>TariqueAnsari</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>279</v>
-      </c>
-      <c r="B10" t="str">
-        <f>REPLACE(A10, 1,3, "Tar")</f>
-        <v>Tarson A</v>
+        <v>299</v>
+      </c>
+      <c r="K10" t="s">
+        <v>288</v>
+      </c>
+      <c r="L10" t="s">
+        <v>289</v>
+      </c>
+      <c r="M10" t="s">
+        <v>290</v>
+      </c>
+      <c r="N10" t="str">
+        <f>_xlfn.TEXTJOIN(" | ",TRUE,K10,L10,M10)</f>
+        <v>aa | aaa | aaaa</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>300</v>
+      </c>
+      <c r="K11" t="s">
+        <v>291</v>
+      </c>
+      <c r="M11" t="s">
+        <v>291</v>
+      </c>
+      <c r="N11" t="str">
+        <f>_xlfn.TEXTJOIN(" | ",TRUE,K11,L11,M11)</f>
+        <v>bbbb | bbbb</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>301</v>
+      </c>
+      <c r="K12" t="s">
+        <v>292</v>
+      </c>
+      <c r="N12" t="str">
+        <f>_xlfn.TEXTJOIN(" | ",TRUE,K12,L12,M12)</f>
+        <v>cccccc</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -4452,7 +4545,7 @@
         <v>9</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -4465,30 +4558,30 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" s="20">
         <f ca="1">TODAY()</f>
-        <v>46231</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="24">
         <f ca="1">NOW()</f>
-        <v>46231.860719444441</v>
+        <v>46234.854374652779</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" s="20">
         <f>DATE(2025, 12,22)</f>
@@ -4501,7 +4594,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7">
         <f>YEAR(B2)</f>
@@ -4510,7 +4603,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B8">
         <f>MONTH(B2)</f>
@@ -4519,7 +4612,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9">
         <f>DAY(B2)</f>
@@ -4528,7 +4621,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B10">
         <f>DATEDIF(B2,C2,"m")</f>
@@ -4537,16 +4630,16 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" s="20">
         <f ca="1">WORKDAY(B4,10)</f>
-        <v>46245</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12" s="18">
         <f>NETWORKDAYS(B2,C2)</f>
@@ -4555,7 +4648,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="20">
         <f>EOMONTH(B2,0)</f>
@@ -4583,30 +4676,30 @@
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.35">
       <c r="O1" t="s">
+        <v>195</v>
+      </c>
+      <c r="P1" t="s">
         <v>196</v>
-      </c>
-      <c r="P1" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="2" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B2" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="F2" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>107</v>
-      </c>
       <c r="O2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P2">
         <v>10</v>
@@ -4628,23 +4721,23 @@
         <v>17</v>
       </c>
       <c r="D3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="F3" s="9">
         <v>25000</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J3">
         <f>SUM(Sales_Amount)</f>
         <v>403400</v>
       </c>
       <c r="O3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P3">
         <v>20</v>
@@ -4666,16 +4759,16 @@
         <v>52</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="F4" s="9">
         <v>55000</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J4">
         <f>COUNT(Sales_Amount)</f>
@@ -4686,7 +4779,7 @@
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="P4">
         <v>14</v>
@@ -4708,23 +4801,23 @@
         <v>17</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F5" s="9">
         <v>23400</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="J5">
         <f>AVERAGE(Sales_Amount)</f>
         <v>40340</v>
       </c>
       <c r="O5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P5">
         <v>20</v>
@@ -4738,23 +4831,23 @@
         <v>54</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F6" s="9">
         <v>22000</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J6">
         <f>SUMIF(C3:C12,"Rahul",Sales_Amount)</f>
         <v>238400</v>
       </c>
       <c r="O6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P6">
         <v>11</v>
@@ -4768,23 +4861,23 @@
         <v>52</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F7" s="9">
         <v>18000</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J7">
         <f>COUNTIF(C3:C12,"Rahul")</f>
         <v>5</v>
       </c>
       <c r="O7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P7">
         <v>12</v>
@@ -4798,19 +4891,19 @@
         <v>17</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F8" s="9">
         <v>60000</v>
       </c>
       <c r="I8" s="49" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="O8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P8">
         <v>12</v>
@@ -4824,16 +4917,16 @@
         <v>17</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="F9" s="13">
         <v>50000</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J9">
         <f>SUMIFS(Sales_Amount,C3:C12,"Rahul",D3:D12,"North")</f>
@@ -4844,7 +4937,7 @@
         <v>75000</v>
       </c>
       <c r="O9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P9">
         <v>19</v>
@@ -4858,19 +4951,19 @@
         <v>52</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>110</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="F10" s="50">
         <v>45000</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="P10">
         <v>13</v>
@@ -4884,19 +4977,19 @@
         <v>17</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F11" s="50">
         <v>80000</v>
       </c>
       <c r="I11" s="49" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="O11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P11">
         <v>20</v>
@@ -4910,10 +5003,10 @@
         <v>54</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F12" s="50">
         <v>25000</v>
@@ -4941,51 +5034,51 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="25" t="s">
-        <v>199</v>
-      </c>
       <c r="C1" s="25" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="E1" s="25" t="s">
         <v>70</v>
       </c>
       <c r="F1" s="25" t="s">
+        <v>199</v>
+      </c>
+      <c r="G1" s="25" t="s">
         <v>200</v>
-      </c>
-      <c r="G1" s="25" t="s">
-        <v>201</v>
       </c>
       <c r="H1" s="25" t="s">
         <v>11</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F2" s="2">
         <v>1</v>
@@ -4997,27 +5090,27 @@
         <v>50000</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>207</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F3" s="2">
         <v>2</v>
@@ -5029,27 +5122,27 @@
         <v>40000</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>54</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="F4" s="2">
         <v>4</v>
@@ -5061,27 +5154,27 @@
         <v>10000</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F5" s="2">
         <v>1</v>
@@ -5093,27 +5186,27 @@
         <v>7000</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>217</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F6" s="2">
         <v>3</v>
@@ -5125,27 +5218,27 @@
         <v>9000</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F7" s="2">
         <v>1</v>
@@ -5157,27 +5250,27 @@
         <v>22000</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>221</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F8" s="2">
         <v>1</v>
@@ -5189,27 +5282,27 @@
         <v>35000</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>223</v>
-      </c>
       <c r="C9" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F9" s="2">
         <v>2</v>
@@ -5221,27 +5314,27 @@
         <v>96000</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="F10" s="2">
         <v>2</v>
@@ -5253,24 +5346,24 @@
         <v>5200</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F11" s="2">
         <v>3</v>
@@ -5282,18 +5375,18 @@
         <v>63000</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D16" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E16" s="51" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="F16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G16" t="s">
         <v>11</v>
@@ -5301,7 +5394,7 @@
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E17" t="str">
         <f>VLOOKUP($D17,$A$1:$I$11,MATCH(E$16,$A$1:$I$1,0),FALSE)</f>
@@ -5318,7 +5411,7 @@
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" ref="E18:G20" si="1">VLOOKUP($D18,$A$1:$I$11,MATCH(E$16,$A$1:$I$1,0),FALSE)</f>
@@ -5335,7 +5428,7 @@
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.35">
       <c r="D19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="1"/>
@@ -5352,7 +5445,7 @@
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.35">
       <c r="D20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E20" t="str">
         <f t="shared" si="1"/>
@@ -5393,48 +5486,48 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>69</v>
       </c>
       <c r="G1" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="H1" s="26" t="s">
         <v>245</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="I1" s="26" t="s">
+        <v>247</v>
+      </c>
+      <c r="P1" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>127</v>
+      </c>
+      <c r="U1" t="s">
         <v>246</v>
-      </c>
-      <c r="I1" s="26" t="s">
-        <v>248</v>
-      </c>
-      <c r="P1" t="s">
-        <v>236</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>128</v>
-      </c>
-      <c r="U1" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>142</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>143</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>11</v>
@@ -5447,26 +5540,26 @@
         <v>44986</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G2" t="s">
         <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I2">
         <v>35000</v>
       </c>
       <c r="K2" s="14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M2" s="2"/>
       <c r="P2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="Q2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="U2" t="s">
         <v>25</v>
@@ -5474,10 +5567,10 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>25</v>
@@ -5490,26 +5583,26 @@
         <v>45031</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G3" t="s">
         <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I3">
         <v>42000</v>
       </c>
       <c r="K3" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M3" s="2"/>
       <c r="P3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Q3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U3" t="s">
         <v>11</v>
@@ -5517,13 +5610,13 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="D4" s="15">
         <f t="shared" ca="1" si="0"/>
@@ -5533,74 +5626,74 @@
         <v>45066</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G4" t="s">
         <v>54</v>
       </c>
       <c r="H4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I4">
         <v>41000</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M4" s="2"/>
       <c r="P4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Q4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>154</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="15">
         <f t="shared" ca="1" si="0"/>
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G5" t="s">
         <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I5">
         <v>48000</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Q5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>157</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>11</v>
@@ -5613,19 +5706,19 @@
         <v>45087</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G6" t="s">
         <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I6">
         <v>39000</v>
       </c>
       <c r="K6" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
@@ -5633,12 +5726,12 @@
         <v>11</v>
       </c>
       <c r="K7" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="K8" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -5681,19 +5774,19 @@
   <sheetData>
     <row r="1" spans="1:61" x14ac:dyDescent="0.35">
       <c r="A1" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="31" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>139</v>
       </c>
       <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P1" s="52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q1" s="52"/>
       <c r="R1" s="52"/>
@@ -5705,7 +5798,7 @@
     </row>
     <row r="2" spans="1:61" x14ac:dyDescent="0.35">
       <c r="A2" s="30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B2" s="30" t="s">
         <v>17</v>
@@ -5717,32 +5810,32 @@
         <v>35000</v>
       </c>
       <c r="F2" s="32" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G2" t="str">
         <f>INDEX(A1:D6,3,2)</f>
         <v>Aisha</v>
       </c>
       <c r="P2" s="47" t="s">
+        <v>260</v>
+      </c>
+      <c r="Q2" s="47" t="s">
         <v>261</v>
       </c>
-      <c r="Q2" s="47" t="s">
-        <v>262</v>
-      </c>
       <c r="R2" s="47" t="s">
+        <v>267</v>
+      </c>
+      <c r="S2" s="47" t="s">
         <v>268</v>
-      </c>
-      <c r="S2" s="47" t="s">
-        <v>269</v>
       </c>
       <c r="T2" s="46"/>
       <c r="BI2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:61" x14ac:dyDescent="0.35">
       <c r="A3" s="30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B3" s="30" t="s">
         <v>52</v>
@@ -5754,7 +5847,7 @@
         <v>42000</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G3">
         <f>MATCH("Rahul",B1:B6,0)</f>
@@ -5767,31 +5860,31 @@
         <v>1.5</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="T3" s="3"/>
       <c r="BI3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:61" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="30" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>54</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D4" s="30">
         <v>50000</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P4" s="3">
         <v>13</v>
@@ -5800,17 +5893,17 @@
         <v>1.555555</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="BI4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:61" x14ac:dyDescent="0.35">
       <c r="A5" s="30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>14</v>
@@ -5826,14 +5919,14 @@
       </c>
       <c r="Q5" s="3"/>
       <c r="R5" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
     </row>
     <row r="6" spans="1:61" x14ac:dyDescent="0.35">
       <c r="A6" s="30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>34</v>
@@ -5849,7 +5942,7 @@
       </c>
       <c r="Q6" s="3"/>
       <c r="R6" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>

</xml_diff>

<commit_message>
Advance sum function and index and match func
</commit_message>
<xml_diff>
--- a/Conditional_Formatting_Practice.xlsx
+++ b/Conditional_Formatting_Practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dmart_sales_7_9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E1A11C-9292-450F-BE88-DCAEE8643B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FE5C92-30F6-4146-8801-EC5A97BE5A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="816" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="816" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conditional_Formatting_Practice" sheetId="1" r:id="rId1"/>
@@ -1000,7 +1000,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -1295,10 +1295,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="20% - Accent2" xfId="1" builtinId="34"/>
@@ -4577,10 +4577,10 @@
       </c>
       <c r="B4" s="20">
         <f ca="1">TODAY()</f>
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F4" s="20"/>
-      <c r="H4" s="53">
+      <c r="H4" s="52">
         <v>1234567</v>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="B11" s="20">
         <f ca="1">WORKDAY(B4,10)</f>
-        <v>46251</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="D5" s="15">
         <f t="shared" ca="1" si="0"/>
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="7" t="s">
@@ -5797,13 +5797,13 @@
       <c r="D1" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="P1" s="52" t="s">
+      <c r="P1" s="53" t="s">
         <v>161</v>
       </c>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
-      <c r="T1" s="52"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53"/>
+      <c r="T1" s="53"/>
       <c r="BI1" t="s">
         <v>2</v>
       </c>

</xml_diff>